<commit_message>
Update source inventory after inspecting rainfall and crop files
</commit_message>
<xml_diff>
--- a/Meghalaya_Source_Inventory_Phase1.xlsx
+++ b/Meghalaya_Source_Inventory_Phase1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Course Work\Artificial Intelligence\assignment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C667523-C9DA-4A57-9EE2-B5E7BE59912F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2865095C-6451-41D1-9DFC-99B40DB62CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="47">
   <si>
     <t>Source / Organization</t>
   </si>
@@ -52,18 +52,6 @@
     <t>Web portal + PDF</t>
   </si>
   <si>
-    <t>English; some Khasi/Garo documents may be available</t>
-  </si>
-  <si>
-    <t>Rainfall reports, Kharif crop reports, agriculture statistics and advisories relevant to rainfall–crop analysis.</t>
-  </si>
-  <si>
-    <t>district, year, season, rainfall, crop, area, production, yield, advisory, source</t>
-  </si>
-  <si>
-    <t>Different documents use different layouts; coverage varies by year/topic; some PDFs may require OCR or table extraction.</t>
-  </si>
-  <si>
     <t>Meghalaya Department of Agriculture – Crop Statistics</t>
   </si>
   <si>
@@ -158,6 +146,21 @@
   </si>
   <si>
     <t>Acts mainly as an index; individual publications must be assessed separately.</t>
+  </si>
+  <si>
+    <t>Web portal + PDF + Scanned PDF</t>
+  </si>
+  <si>
+    <t>English; some Khasi/Garo documents available</t>
+  </si>
+  <si>
+    <t>Provides station-wise monthly rainfall data and district-wise Kharif crop statistics. Rainfall data can be linked with crop area, production, and yield for rainfall–crop analysis</t>
+  </si>
+  <si>
+    <t>year, month, district, station, rainfall_mm, rainy_days, crop_year, season, crop_name, area, production, yield</t>
+  </si>
+  <si>
+    <t>Rainfall Excel contains some missing station/month observations and requires restructuring. The crop report is a scanned image PDF with no embedded text layer, so OCR and table extraction are required.</t>
   </si>
 </sst>
 </file>
@@ -660,157 +663,157 @@
         <v>8</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>9</v>
+        <v>42</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="54.45" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C3" s="9" t="s">
         <v>9</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="54.45" customHeight="1">
       <c r="A4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="G4" s="1" t="s">
         <v>21</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="54.45" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>9</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="54.45" customHeight="1">
       <c r="A6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="G6" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="54.45" customHeight="1">
       <c r="A7" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="54.45" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>9</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>